<commit_message>
Added Bug Ticket column to mention HERESUP tickets on dashboard
</commit_message>
<xml_diff>
--- a/data/Error_Count_Diff_P172_vs_P173_EU.xlsx
+++ b/data/Error_Count_Diff_P172_vs_P173_EU.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mghate\Downloads\Automation\EU\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mghate\Downloads\GitHub\diff-dashboard\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD8028DC-52E7-402B-AC44-C92CEE18F5B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FBC3DFA-D4BC-4ABD-A799-2CD604954319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="142">
   <si>
     <t>testId</t>
   </si>
@@ -311,16 +311,159 @@
   </si>
   <si>
     <t>STABLE_NAMED_OBJECT_IDS_LOCALLY</t>
+  </si>
+  <si>
+    <t>Bug Ticket</t>
+  </si>
+  <si>
+    <t>HERESUP-8187</t>
+  </si>
+  <si>
+    <t>HERESUP-35609</t>
+  </si>
+  <si>
+    <t>HERESUP-35608</t>
+  </si>
+  <si>
+    <t>HERESUP-64253</t>
+  </si>
+  <si>
+    <t>HERESUP-8241</t>
+  </si>
+  <si>
+    <t>HERESUP-8215</t>
+  </si>
+  <si>
+    <t>HERESUP-12216</t>
+  </si>
+  <si>
+    <t>HERESUP-8207</t>
+  </si>
+  <si>
+    <t>HERESUP-8221</t>
+  </si>
+  <si>
+    <t>HERESUP-8336</t>
+  </si>
+  <si>
+    <t>HERESUP-8186</t>
+  </si>
+  <si>
+    <t>HERESUP-8188</t>
+  </si>
+  <si>
+    <t>HERESUP-8192</t>
+  </si>
+  <si>
+    <t>HERESUP-35611</t>
+  </si>
+  <si>
+    <t>HERESUP-34067</t>
+  </si>
+  <si>
+    <t>HERESUP-8208</t>
+  </si>
+  <si>
+    <t>NO TICKET</t>
+  </si>
+  <si>
+    <t>HERESUP-8199</t>
+  </si>
+  <si>
+    <t>HERESUP-8198</t>
+  </si>
+  <si>
+    <t>HERESUP-8240</t>
+  </si>
+  <si>
+    <t>HERESUP-8226</t>
+  </si>
+  <si>
+    <t>HERESUP-8233</t>
+  </si>
+  <si>
+    <t>HERESUP-8231</t>
+  </si>
+  <si>
+    <t>HERESUP-8227</t>
+  </si>
+  <si>
+    <t>HERESUP-8228</t>
+  </si>
+  <si>
+    <t>HERESUP-8232</t>
+  </si>
+  <si>
+    <t>HERESUP-8229</t>
+  </si>
+  <si>
+    <t>HERESUP-8230</t>
+  </si>
+  <si>
+    <t>HERESUP-8926</t>
+  </si>
+  <si>
+    <t>HERESUP-8239</t>
+  </si>
+  <si>
+    <t>HERESUP-35615</t>
+  </si>
+  <si>
+    <t>HERESUP-21393</t>
+  </si>
+  <si>
+    <t>HERESUP-8196</t>
+  </si>
+  <si>
+    <t>HERESUP-8200</t>
+  </si>
+  <si>
+    <t>HERESUP-8197</t>
+  </si>
+  <si>
+    <t>HERESUP-57439</t>
+  </si>
+  <si>
+    <t>HERESUP-35614</t>
+  </si>
+  <si>
+    <t>HERESUP-8180</t>
+  </si>
+  <si>
+    <t>HERESUP-8182</t>
+  </si>
+  <si>
+    <t>HERESUP-60308</t>
+  </si>
+  <si>
+    <t>HERESUP-8184</t>
+  </si>
+  <si>
+    <t>HERESUP-8245</t>
+  </si>
+  <si>
+    <t>HERESUP-8178</t>
+  </si>
+  <si>
+    <t>HERESUP-8165</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -346,13 +489,48 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -667,7 +845,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:H45"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.109375" bestFit="1" customWidth="1"/>
@@ -675,9 +853,10 @@
     <col min="3" max="4" width="8.33203125" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="14.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -699,8 +878,11 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H1" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -722,8 +904,11 @@
       <c r="G2">
         <v>13</v>
       </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H2" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>10</v>
       </c>
@@ -745,8 +930,11 @@
       <c r="G3">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H3" s="2" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>12</v>
       </c>
@@ -768,8 +956,11 @@
       <c r="G4">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H4" s="2" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>14</v>
       </c>
@@ -791,8 +982,11 @@
       <c r="G5">
         <v>1</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H5" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -814,8 +1008,11 @@
       <c r="G6">
         <v>-966</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H6" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>19</v>
       </c>
@@ -837,8 +1034,11 @@
       <c r="G7">
         <v>-52</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H7" s="2" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>21</v>
       </c>
@@ -860,8 +1060,11 @@
       <c r="G8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H8" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -883,8 +1086,11 @@
       <c r="G9">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H9" s="1" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -906,8 +1112,11 @@
       <c r="G10">
         <v>-33</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H10" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>27</v>
       </c>
@@ -929,8 +1138,11 @@
       <c r="G11">
         <v>331</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H11" s="1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -952,8 +1164,11 @@
       <c r="G12">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H12" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>31</v>
       </c>
@@ -975,8 +1190,11 @@
       <c r="G13">
         <v>-9</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H13" s="1" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>33</v>
       </c>
@@ -998,8 +1216,11 @@
       <c r="G14">
         <v>92</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H14" s="1" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>35</v>
       </c>
@@ -1021,8 +1242,11 @@
       <c r="G15">
         <v>0</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H15" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -1044,8 +1268,11 @@
       <c r="G16">
         <v>0</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H16" s="2" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>39</v>
       </c>
@@ -1067,8 +1294,11 @@
       <c r="G17">
         <v>0</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H17" s="1" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>41</v>
       </c>
@@ -1090,8 +1320,11 @@
       <c r="G18">
         <v>1343</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H18" s="2" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>43</v>
       </c>
@@ -1113,8 +1346,11 @@
       <c r="G19">
         <v>571</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H19" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>45</v>
       </c>
@@ -1136,8 +1372,11 @@
       <c r="G20">
         <v>4</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H20" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>47</v>
       </c>
@@ -1159,8 +1398,11 @@
       <c r="G21">
         <v>3853</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H21" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>49</v>
       </c>
@@ -1182,8 +1424,11 @@
       <c r="G22">
         <v>-5</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H22" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>51</v>
       </c>
@@ -1205,8 +1450,11 @@
       <c r="G23">
         <v>1</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H23" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>53</v>
       </c>
@@ -1228,8 +1476,11 @@
       <c r="G24">
         <v>-3</v>
       </c>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H24" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>55</v>
       </c>
@@ -1251,8 +1502,11 @@
       <c r="G25">
         <v>10</v>
       </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H25" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>57</v>
       </c>
@@ -1274,8 +1528,11 @@
       <c r="G26">
         <v>-1</v>
       </c>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H26" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>59</v>
       </c>
@@ -1297,8 +1554,11 @@
       <c r="G27">
         <v>23</v>
       </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H27" s="1" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>61</v>
       </c>
@@ -1320,8 +1580,11 @@
       <c r="G28">
         <v>157</v>
       </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H28" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>63</v>
       </c>
@@ -1343,8 +1606,11 @@
       <c r="G29">
         <v>112</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H29" s="1" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>65</v>
       </c>
@@ -1366,8 +1632,11 @@
       <c r="G30">
         <v>2</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H30" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>67</v>
       </c>
@@ -1389,8 +1658,11 @@
       <c r="G31">
         <v>3545</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H31" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>69</v>
       </c>
@@ -1412,8 +1684,11 @@
       <c r="G32">
         <v>0</v>
       </c>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H32" s="2" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>71</v>
       </c>
@@ -1435,8 +1710,11 @@
       <c r="G33">
         <v>0</v>
       </c>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H33" s="1" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>73</v>
       </c>
@@ -1458,8 +1736,11 @@
       <c r="G34">
         <v>0</v>
       </c>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H34" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>75</v>
       </c>
@@ -1481,8 +1762,11 @@
       <c r="G35">
         <v>8</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H35" s="1" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>77</v>
       </c>
@@ -1504,8 +1788,11 @@
       <c r="G36">
         <v>1</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H36" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>79</v>
       </c>
@@ -1527,8 +1814,11 @@
       <c r="G37">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H37" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>81</v>
       </c>
@@ -1550,8 +1840,11 @@
       <c r="G38">
         <v>0</v>
       </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H38" s="2" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>83</v>
       </c>
@@ -1573,8 +1866,11 @@
       <c r="G39">
         <v>-2</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H39" s="1" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>85</v>
       </c>
@@ -1596,8 +1892,11 @@
       <c r="G40">
         <v>-15</v>
       </c>
-    </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H40" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>87</v>
       </c>
@@ -1619,8 +1918,11 @@
       <c r="G41">
         <v>-10</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H41" s="2" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>89</v>
       </c>
@@ -1642,8 +1944,11 @@
       <c r="G42">
         <v>1037</v>
       </c>
-    </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H42" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>91</v>
       </c>
@@ -1665,8 +1970,11 @@
       <c r="G43">
         <v>3</v>
       </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H43" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>93</v>
       </c>
@@ -1688,8 +1996,11 @@
       <c r="G44">
         <v>-9</v>
       </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="H44" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>95</v>
       </c>
@@ -1711,14 +2022,31 @@
       <c r="G45">
         <v>-4943</v>
       </c>
+      <c r="H45" s="2" t="s">
+        <v>141</v>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G45">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="5" priority="5" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="4" priority="6" operator="greaterThan">
       <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H45">
+    <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
+      <formula>"Not started"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="2" operator="equal">
+      <formula>"Not executed"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="3" operator="equal">
+      <formula>"Fail"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="4" operator="equal">
+      <formula>"Pass"</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>